<commit_message>
Arreglos de importación y exportación de data panel admin
</commit_message>
<xml_diff>
--- a/catalogo_vehiculos.xlsx
+++ b/catalogo_vehiculos.xlsx
@@ -1,23 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://camalmusalem.sharepoint.com/sites/TOYOTA_MUSALEM/MUSALEM/VENTAS/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="185" documentId="13_ncr:1_{85358A0F-780A-44E9-85C9-0C2D4A1575D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA4FF0DA-99DA-4AB4-8710-9453510ED53D}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Catálogo vehículos" sheetId="1" r:id="rId4"/>
+    <sheet name="Catálogo vehículos" sheetId="1" r:id="rId1"/>
+    <sheet name="Catalogo Vehiculos Seminuevos" sheetId="2" r:id="rId2"/>
+    <sheet name="Catalogo Repuestos" sheetId="3" r:id="rId3"/>
+    <sheet name="Catalogo Accesorios" sheetId="5" r:id="rId4"/>
+    <sheet name="Catalogo Merch" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catálogo vehículos'!$A$1:$CA$1</definedName>
   </definedNames>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="332">
   <si>
     <t>ID</t>
   </si>
@@ -728,31 +751,324 @@
   </si>
   <si>
     <t>Blanco Perlado, Rojo Emoción, Negro Montecarlo</t>
+  </si>
+  <si>
+    <t>VU</t>
+  </si>
+  <si>
+    <t>BMW</t>
+  </si>
+  <si>
+    <t>Codigo Interno</t>
+  </si>
+  <si>
+    <t>Nombre Repuesto</t>
+  </si>
+  <si>
+    <t>Precio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compatible con </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disponible  en </t>
+  </si>
+  <si>
+    <t>ACEITE SN C2 5W - 30 BIDON 4L</t>
+  </si>
+  <si>
+    <t>Sucursal La Serena / Sucursal Ovalle</t>
+  </si>
+  <si>
+    <t>BATERIA YUASA  40B19L  (35 AMP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sucursal La Serena </t>
+  </si>
+  <si>
+    <t>Fotografia</t>
+  </si>
+  <si>
+    <t>Precio Oferta</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Sucursal Ovalle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corolla Cross- Corolla Sedan - Yaris Sedan </t>
+  </si>
+  <si>
+    <t>Nombre Merch</t>
+  </si>
+  <si>
+    <t>BILLETERA  GR X</t>
+  </si>
+  <si>
+    <t>Talla</t>
+  </si>
+  <si>
+    <t>POLERA GR POLO BLANCA</t>
+  </si>
+  <si>
+    <t>S - XL</t>
+  </si>
+  <si>
+    <t>X1 SDRIVE18D 2.0 AT</t>
+  </si>
+  <si>
+    <t>Bono Financiaminto</t>
+  </si>
+  <si>
+    <t>Precio Lista + Bono Financiaminto</t>
+  </si>
+  <si>
+    <t>2  WD</t>
+  </si>
+  <si>
+    <t>Tipo Combustible</t>
+  </si>
+  <si>
+    <t>Diesel</t>
+  </si>
+  <si>
+    <t>KM</t>
+  </si>
+  <si>
+    <t>SEGURIDAD</t>
+  </si>
+  <si>
+    <t>Sistema de frenos ABS</t>
+  </si>
+  <si>
+    <t>Distribución electrónica de frenado (EBD)</t>
+  </si>
+  <si>
+    <t>Asistencia de frenado de emergencia (BA)</t>
+  </si>
+  <si>
+    <t>Control de estabilidad ESP / VSC</t>
+  </si>
+  <si>
+    <t>Control de tracción (TCS / TRC)</t>
+  </si>
+  <si>
+    <t>Control de estabilidad del remolque (TSC)</t>
+  </si>
+  <si>
+    <t>Asistente de arranque en pendiente (HAC)</t>
+  </si>
+  <si>
+    <t>Asistente de descenso (DAC)</t>
+  </si>
+  <si>
+    <t>Diferencial electrónico (e-LSD)</t>
+  </si>
+  <si>
+    <t>Dirección asistida eléctrica con control de estabilidad</t>
+  </si>
+  <si>
+    <t>Frenos de disco ventilados (delanteros/traseros)</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Mantenciones</t>
+  </si>
+  <si>
+    <t>Potencia</t>
+  </si>
+  <si>
+    <t>Torque</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>mandos al volante</t>
+  </si>
+  <si>
+    <t>camara de retroceso</t>
+  </si>
+  <si>
+    <t>bluetooth</t>
+  </si>
+  <si>
+    <t>android auto</t>
+  </si>
+  <si>
+    <t>apple car play</t>
+  </si>
+  <si>
+    <t>sensores de retroceso</t>
+  </si>
+  <si>
+    <t>neblineros</t>
+  </si>
+  <si>
+    <t>llantas de aleación</t>
+  </si>
+  <si>
+    <t>espejos electricos</t>
+  </si>
+  <si>
+    <t>techo panoramico</t>
+  </si>
+  <si>
+    <t>aire acondicionado</t>
+  </si>
+  <si>
+    <t>dos copias de llave</t>
+  </si>
+  <si>
+    <t>numero de puertas</t>
+  </si>
+  <si>
+    <t>numero de propietarios</t>
+  </si>
+  <si>
+    <t>Certificación  Toyota Usados</t>
+  </si>
+  <si>
+    <t>climatizador / bi-zona</t>
+  </si>
+  <si>
+    <t>Descripcion corta</t>
+  </si>
+  <si>
+    <t>Descripcion tecnica</t>
+  </si>
+  <si>
+    <t>Categoria principal</t>
+  </si>
+  <si>
+    <t>Subcategoria</t>
+  </si>
+  <si>
+    <t>GR</t>
+  </si>
+  <si>
+    <t>Descripción tecnica</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Mantenimiento</t>
+  </si>
+  <si>
+    <t>Tiempo estimado de entrega</t>
+  </si>
+  <si>
+    <t>TOYOTA</t>
+  </si>
+  <si>
+    <t>COROLLA SEDAN 1.8 HIBRIDO</t>
+  </si>
+  <si>
+    <t>Año vehiculo compatible</t>
+  </si>
+  <si>
+    <t>2020 al 2026</t>
+  </si>
+  <si>
+    <t>Inventario / stok</t>
+  </si>
+  <si>
+    <t>a pedido</t>
+  </si>
+  <si>
+    <t>disponible</t>
+  </si>
+  <si>
+    <t>5 dias</t>
+  </si>
+  <si>
+    <t>inmediata</t>
+  </si>
+  <si>
+    <t>Precio instalado</t>
+  </si>
+  <si>
+    <t>merch</t>
+  </si>
+  <si>
+    <t>accesorio</t>
+  </si>
+  <si>
+    <t>Blanco Perlado Platinum</t>
+  </si>
+  <si>
+    <t>Automovil</t>
+  </si>
+  <si>
+    <t>2 WD</t>
+  </si>
+  <si>
+    <t>Hibrido</t>
+  </si>
+  <si>
+    <t>LLANTA ALEACION 18´ GR HILUX</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Compatibilidad</t>
+  </si>
+  <si>
+    <t>CUBRE CARTER RAIZE</t>
+  </si>
+  <si>
+    <t>2021-2026</t>
+  </si>
+  <si>
+    <t>La Serena</t>
+  </si>
+  <si>
+    <t>Carroceria</t>
+  </si>
+  <si>
+    <t>Blanco</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$$-340A]#,##0"/>
+  </numFmts>
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -769,7 +1085,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -792,21 +1108,113 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+  <cellXfs count="14">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -1096,95 +1504,82 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CA14"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.141" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="11.711" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="31.707" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="17" max="17" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="18" max="18" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="19" max="19" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="20" max="20" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="21" max="21" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="22" max="22" width="52.987" bestFit="true" customWidth="true" style="0"/>
-    <col min="23" max="23" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="24" max="24" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="25" max="25" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="26" max="26" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="27" max="27" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="28" max="28" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="29" max="29" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="30" max="30" width="43.561" bestFit="true" customWidth="true" style="0"/>
-    <col min="31" max="31" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="32" max="32" width="26.993" bestFit="true" customWidth="true" style="0"/>
-    <col min="33" max="33" width="32.849" bestFit="true" customWidth="true" style="0"/>
-    <col min="34" max="34" width="32.849" bestFit="true" customWidth="true" style="0"/>
-    <col min="35" max="35" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="36" max="36" width="32.849" bestFit="true" customWidth="true" style="0"/>
-    <col min="37" max="37" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="38" max="38" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="39" max="39" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="40" max="40" width="25.851" bestFit="true" customWidth="true" style="0"/>
-    <col min="41" max="41" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="42" max="42" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="43" max="43" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="44" max="44" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="45" max="45" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="46" max="46" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="47" max="47" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="48" max="48" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="49" max="49" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="50" max="50" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="51" max="51" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="52" max="52" width="15.282" bestFit="true" customWidth="true" style="0"/>
-    <col min="53" max="53" width="19.995" bestFit="true" customWidth="true" style="0"/>
-    <col min="54" max="54" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="55" max="55" width="32.849" bestFit="true" customWidth="true" style="0"/>
-    <col min="56" max="56" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="57" max="57" width="30.564" bestFit="true" customWidth="true" style="0"/>
-    <col min="58" max="58" width="34.135" bestFit="true" customWidth="true" style="0"/>
-    <col min="59" max="59" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="60" max="60" width="29.421" bestFit="true" customWidth="true" style="0"/>
-    <col min="61" max="61" width="22.28" bestFit="true" customWidth="true" style="0"/>
-    <col min="62" max="62" width="32.849" bestFit="true" customWidth="true" style="0"/>
-    <col min="63" max="63" width="28.136" bestFit="true" customWidth="true" style="0"/>
-    <col min="64" max="64" width="67.127" bestFit="true" customWidth="true" style="0"/>
-    <col min="65" max="65" width="155.676" bestFit="true" customWidth="true" style="0"/>
-    <col min="66" max="66" width="97.833" bestFit="true" customWidth="true" style="0"/>
-    <col min="67" max="67" width="63.556" bestFit="true" customWidth="true" style="0"/>
-    <col min="68" max="68" width="63.556" bestFit="true" customWidth="true" style="0"/>
-    <col min="69" max="69" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="70" max="70" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="71" max="71" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="72" max="72" width="375.051" bestFit="true" customWidth="true" style="0"/>
-    <col min="73" max="73" width="267.649" bestFit="true" customWidth="true" style="0"/>
-    <col min="74" max="74" width="284.216" bestFit="true" customWidth="true" style="0"/>
-    <col min="75" max="75" width="123.827" bestFit="true" customWidth="true" style="0"/>
-    <col min="76" max="76" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="77" max="77" width="244.083" bestFit="true" customWidth="true" style="0"/>
-    <col min="78" max="78" width="101.404" bestFit="true" customWidth="true" style="0"/>
-    <col min="79" max="79" width="135.538" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="53" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="43.5546875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="27" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="20" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="41" max="42" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="20" bestFit="1" customWidth="1"/>
+    <col min="46" max="47" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="51" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="20" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="30.5546875" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="34.109375" bestFit="1" customWidth="1"/>
+    <col min="59" max="60" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="67.109375" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="155.6640625" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="97.6640625" bestFit="1" customWidth="1"/>
+    <col min="67" max="68" width="63.5546875" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="70" max="71" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="72" max="72" width="375" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="267.6640625" bestFit="1" customWidth="1"/>
+    <col min="74" max="74" width="284.33203125" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="123.6640625" bestFit="1" customWidth="1"/>
+    <col min="76" max="76" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="77" max="77" width="244.109375" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="101.44140625" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="135.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:79">
+    <row r="1" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1423,7 +1818,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:79">
+    <row r="2" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1554,7 +1949,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="3" spans="1:79">
+    <row r="3" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1694,7 +2089,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:79">
+    <row r="4" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1750,7 +2145,7 @@
         <v>5</v>
       </c>
       <c r="BE4">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="BF4">
         <v>21.3</v>
@@ -1780,7 +2175,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="1:79">
+    <row r="5" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1857,10 +2252,10 @@
         <v>227</v>
       </c>
       <c r="AT5">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="AU5">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="AY5">
         <v>2750</v>
@@ -1914,7 +2309,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:79">
+    <row r="6" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2054,7 +2449,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:79">
+    <row r="7" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2179,7 +2574,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="8" spans="1:79">
+    <row r="8" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2256,7 +2651,7 @@
         <v>1980</v>
       </c>
       <c r="AT8">
-        <v>32.0</v>
+        <v>32</v>
       </c>
       <c r="AY8">
         <v>3100</v>
@@ -2310,7 +2705,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="9" spans="1:79">
+    <row r="9" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2423,7 +2818,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:79">
+    <row r="10" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2485,7 +2880,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="11" spans="1:79">
+    <row r="11" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2613,7 +3008,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="12" spans="1:79">
+    <row r="12" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2672,10 +3067,10 @@
         <v>453</v>
       </c>
       <c r="AL12">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="AM12">
-        <v>150.0</v>
+        <v>150</v>
       </c>
       <c r="AN12" t="s">
         <v>207</v>
@@ -2717,7 +3112,7 @@
         <v>0</v>
       </c>
       <c r="BI12">
-        <v>5.1</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="BL12" t="s">
         <v>91</v>
@@ -2762,7 +3157,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="13" spans="1:79">
+    <row r="13" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2890,7 +3285,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="14" spans="1:79">
+    <row r="14" spans="1:79" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3022,9 +3417,979 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CA1"/>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <autoFilter ref="A1:CA1" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B472A78-6040-4417-9FF2-B80F382D48B0}">
+  <dimension ref="A1:AU4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" style="3" customWidth="1"/>
+    <col min="3" max="4" width="31.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="22.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="17.109375" style="3" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" style="3" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="5" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="6.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="38.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="38.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="29.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="28.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="38.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="39.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="26.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="28.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="48.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="44.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="19" style="3" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="13.109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="20.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="10.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="17.5546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="40" max="41" width="17" style="3" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="17.88671875" style="3" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="27.33203125" style="3" customWidth="1"/>
+    <col min="44" max="44" width="23.109375" style="3" customWidth="1"/>
+    <col min="45" max="45" width="27.6640625" style="3" customWidth="1"/>
+    <col min="46" max="46" width="18" style="3" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="22.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="48" max="16384" width="11.5546875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="U1" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="13"/>
+      <c r="AB1" s="11"/>
+      <c r="AC1" s="12"/>
+      <c r="AD1" s="12"/>
+      <c r="AE1" s="12"/>
+      <c r="AF1" s="11"/>
+      <c r="AG1" s="12"/>
+      <c r="AH1" s="12"/>
+      <c r="AI1" s="12"/>
+      <c r="AJ1" s="11"/>
+      <c r="AK1" s="12"/>
+      <c r="AL1" s="12"/>
+      <c r="AM1" s="12"/>
+      <c r="AN1" s="11"/>
+      <c r="AO1" s="12"/>
+      <c r="AP1" s="12"/>
+      <c r="AQ1" s="12"/>
+      <c r="AR1" s="11"/>
+      <c r="AS1" s="12"/>
+      <c r="AT1" s="12"/>
+      <c r="AU1" s="12"/>
+    </row>
+    <row r="2" spans="1:47" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K2" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="L2" s="8" t="s">
+        <v>260</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="S2" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="T2" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="U2" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="V2" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="W2" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="X2" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="Y2" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="Z2" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="AA2" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="AB2" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="AC2" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="AD2" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="AE2" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="AF2" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="AG2" s="10" t="s">
+        <v>284</v>
+      </c>
+      <c r="AH2" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="AI2" s="10" t="s">
+        <v>286</v>
+      </c>
+      <c r="AJ2" s="10" t="s">
+        <v>287</v>
+      </c>
+      <c r="AK2" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="AL2" s="10" t="s">
+        <v>289</v>
+      </c>
+      <c r="AM2" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="AN2" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="AO2" s="10" t="s">
+        <v>292</v>
+      </c>
+      <c r="AP2" s="10" t="s">
+        <v>293</v>
+      </c>
+      <c r="AQ2" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="AR2" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="AS2" s="10" t="s">
+        <v>294</v>
+      </c>
+      <c r="AT2" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="AU2" s="10" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="3" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>915</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D3" s="3">
+        <v>2022</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>331</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I3" s="3">
+        <v>2022</v>
+      </c>
+      <c r="J3" s="5">
+        <v>25500000</v>
+      </c>
+      <c r="K3" s="5">
+        <v>2000000</v>
+      </c>
+      <c r="L3" s="5">
+        <f>J3-K3</f>
+        <v>23500000</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="P3" s="3">
+        <v>20000</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="T3" s="9">
+        <v>84391</v>
+      </c>
+    </row>
+    <row r="4" spans="1:47" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>838</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="D4" s="3">
+        <v>2024</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="I4" s="3">
+        <v>2024</v>
+      </c>
+      <c r="J4" s="5">
+        <v>21990000</v>
+      </c>
+      <c r="K4" s="5">
+        <v>500000</v>
+      </c>
+      <c r="L4" s="5">
+        <f>J4-K4</f>
+        <v>21490000</v>
+      </c>
+      <c r="N4" t="s">
+        <v>322</v>
+      </c>
+      <c r="O4" t="s">
+        <v>184</v>
+      </c>
+      <c r="P4" s="3">
+        <v>18000</v>
+      </c>
+      <c r="S4" t="s">
+        <v>323</v>
+      </c>
+      <c r="T4" s="3">
+        <v>2125</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="AR1:AU1"/>
+    <mergeCell ref="U1:AA1"/>
+    <mergeCell ref="AB1:AE1"/>
+    <mergeCell ref="AF1:AI1"/>
+    <mergeCell ref="AJ1:AM1"/>
+    <mergeCell ref="AN1:AQ1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA30E8C-0FED-4711-BABC-6B27D5D8B30D}">
+  <dimension ref="A1:N4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="32.109375" style="3" customWidth="1"/>
+    <col min="3" max="4" width="25.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="15.88671875" style="3" customWidth="1"/>
+    <col min="11" max="12" width="39.33203125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="33.5546875" style="3" customWidth="1"/>
+    <col min="14" max="14" width="25.109375" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="11.5546875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>13533</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E2" s="5">
+        <v>35800</v>
+      </c>
+      <c r="F2" s="5">
+        <v>30000</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>40159</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E3" s="5">
+        <v>66283</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M4" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" verticalDpi="0" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7384AA83-A9DD-4F24-A439-EA7A9149A1A4}">
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.44140625" style="3" customWidth="1"/>
+    <col min="2" max="2" width="32.109375" style="3" customWidth="1"/>
+    <col min="3" max="4" width="25.6640625" style="3" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="10" width="15.88671875" style="3" customWidth="1"/>
+    <col min="11" max="12" width="39.33203125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="33.5546875" style="3" customWidth="1"/>
+    <col min="14" max="14" width="25.109375" style="3" customWidth="1"/>
+    <col min="15" max="16384" width="11.5546875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="N1" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>47755</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="I2" s="9" t="s">
+        <v>314</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>328</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>45076</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>327</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7111EA82-C57A-4F6C-B143-22A7D401730B}">
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="15.33203125" style="3" customWidth="1"/>
+    <col min="2" max="3" width="25" style="3" customWidth="1"/>
+    <col min="4" max="8" width="13.5546875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="3"/>
+    <col min="10" max="11" width="17" style="3" customWidth="1"/>
+    <col min="12" max="12" width="22.33203125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="21.109375" style="3" customWidth="1"/>
+    <col min="14" max="16384" width="11.5546875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>45532</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="I2" s="5">
+        <v>35546</v>
+      </c>
+      <c r="J2" s="5">
+        <v>25000</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>46524</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="I3" s="5">
+        <v>21416</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100901A1BAE2DE7AF42A88364D49125E130" ma:contentTypeVersion="14" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="5be12113553bba202029f98c88c16927">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4a8b8af4-029c-4d1b-a237-328becbf44c6" xmlns:ns3="6ac10914-d494-4ee3-afe6-e55ab09badb0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c11e6a1f41e3dda690d86b3021c8b29" ns2:_="" ns3:_="">
+    <xsd:import namespace="4a8b8af4-029c-4d1b-a237-328becbf44c6"/>
+    <xsd:import namespace="6ac10914-d494-4ee3-afe6-e55ab09badb0"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="4a8b8af4-029c-4d1b-a237-328becbf44c6" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8a6ac71b-eadb-4f9d-9a96-155308d405ec" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:description="" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="21" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="6ac10914-d494-4ee3-afe6-e55ab09badb0" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{dccb7a6c-ba98-45fb-8916-486a97d19a94}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="6ac10914-d494-4ee3-afe6-e55ab09badb0">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="6ac10914-d494-4ee3-afe6-e55ab09badb0" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4a8b8af4-029c-4d1b-a237-328becbf44c6">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{521CD37B-0A61-4FFB-B40A-42B45E5339EC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4a8b8af4-029c-4d1b-a237-328becbf44c6"/>
+    <ds:schemaRef ds:uri="6ac10914-d494-4ee3-afe6-e55ab09badb0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F50B43BE-051B-4284-ACD8-69355E07A325}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83D286CF-F72C-4762-B5B3-BCDDF9903DA4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6ac10914-d494-4ee3-afe6-e55ab09badb0"/>
+    <ds:schemaRef ds:uri="4a8b8af4-029c-4d1b-a237-328becbf44c6"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>